<commit_message>
Improved Job shop section
</commit_message>
<xml_diff>
--- a/benchmarks/resultsv8/dentist-general.xlsx
+++ b/benchmarks/resultsv8/dentist-general.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="35">
   <si>
     <t>instances/size-1</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>SATISFIABLE</t>
+  </si>
+  <si>
+    <t>UNKNOWN</t>
   </si>
   <si>
     <t>rules</t>
@@ -507,7 +510,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -516,7 +519,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -525,7 +528,7 @@
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
@@ -533,7 +536,7 @@
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -541,7 +544,7 @@
       <c r="AG1" s="1"/>
       <c r="AH1" s="1"/>
       <c r="AI1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AJ1" s="1"/>
       <c r="AK1" s="1"/>
@@ -561,16 +564,16 @@
         <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>19</v>
@@ -582,16 +585,16 @@
         <v>21</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>19</v>
@@ -603,16 +606,16 @@
         <v>21</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>19</v>
@@ -621,16 +624,16 @@
         <v>20</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>19</v>
@@ -639,16 +642,16 @@
         <v>20</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AH2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AI2" s="1" t="s">
         <v>19</v>
@@ -657,16 +660,16 @@
         <v>20</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AM2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:40">
@@ -816,13 +819,23 @@
       <c r="B4" s="1">
         <v>1200</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+      <c r="C4" s="1">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>198.971</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
       <c r="H4" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="1">
         <v>6.9</v>
@@ -3063,7 +3076,7 @@
   <sheetData>
     <row r="1" spans="1:40">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
@@ -3075,7 +3088,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -3084,7 +3097,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -3093,7 +3106,7 @@
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
@@ -3101,7 +3114,7 @@
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -3109,7 +3122,7 @@
       <c r="AG1" s="1"/>
       <c r="AH1" s="1"/>
       <c r="AI1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AJ1" s="1"/>
       <c r="AK1" s="1"/>
@@ -3119,7 +3132,7 @@
     </row>
     <row r="2" spans="1:40">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>19</v>
@@ -3131,16 +3144,16 @@
         <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>19</v>
@@ -3152,16 +3165,16 @@
         <v>21</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>19</v>
@@ -3173,16 +3186,16 @@
         <v>21</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>19</v>
@@ -3191,16 +3204,16 @@
         <v>20</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>19</v>
@@ -3209,16 +3222,16 @@
         <v>20</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AH2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AI2" s="1" t="s">
         <v>19</v>
@@ -3227,16 +3240,16 @@
         <v>20</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AM2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:40">
@@ -3399,11 +3412,23 @@
         <f t="array" ref="B4">_xlfn.SWITCH($A$2,"average", AVERAGE(Instances!B4:Instances!B4),"median", MEDIAN(Instances!B4:Instances!B4),"min", MIN(Instances!B4:Instances!B4),"max", MAX(Instances!B4:Instances!B4),"diff", MAX(Instances!B4:Instances!B4)-MIN(Instances!B4:Instances!B4))</f>
         <v>0</v>
       </c>
-      <c r="C4" s="1"/>
+      <c r="C4" s="1" cm="1">
+        <f t="array" ref="C4">_xlfn.SWITCH($A$2,"average", AVERAGE(Instances!C4:Instances!C4),"median", MEDIAN(Instances!C4:Instances!C4),"min", MIN(Instances!C4:Instances!C4),"max", MAX(Instances!C4:Instances!C4),"diff", MAX(Instances!C4:Instances!C4)-MIN(Instances!C4:Instances!C4))</f>
+        <v>0</v>
+      </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+      <c r="E4" s="1" cm="1">
+        <f t="array" ref="E4">_xlfn.SWITCH($A$2,"average", AVERAGE(Instances!E4:Instances!E4),"median", MEDIAN(Instances!E4:Instances!E4),"min", MIN(Instances!E4:Instances!E4),"max", MAX(Instances!E4:Instances!E4),"diff", MAX(Instances!E4:Instances!E4)-MIN(Instances!E4:Instances!E4))</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="1" cm="1">
+        <f t="array" ref="F4">_xlfn.SWITCH($A$2,"average", AVERAGE(Instances!F4:Instances!F4),"median", MEDIAN(Instances!F4:Instances!F4),"min", MIN(Instances!F4:Instances!F4),"max", MAX(Instances!F4:Instances!F4),"diff", MAX(Instances!F4:Instances!F4)-MIN(Instances!F4:Instances!F4))</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="1" cm="1">
+        <f t="array" ref="G4">_xlfn.SWITCH($A$2,"average", AVERAGE(Instances!G4:Instances!G4),"median", MEDIAN(Instances!G4:Instances!G4),"min", MIN(Instances!G4:Instances!G4),"max", MAX(Instances!G4:Instances!G4),"diff", MAX(Instances!G4:Instances!G4)-MIN(Instances!G4:Instances!G4))</f>
+        <v>0</v>
+      </c>
       <c r="H4" s="1" cm="1">
         <f t="array" ref="H4">_xlfn.SWITCH($A$2,"average", AVERAGE(Instances!H4:Instances!H4),"median", MEDIAN(Instances!H4:Instances!H4),"min", MIN(Instances!H4:Instances!H4),"max", MAX(Instances!H4:Instances!H4),"diff", MAX(Instances!H4:Instances!H4)-MIN(Instances!H4:Instances!H4))</f>
         <v>0</v>
@@ -5765,7 +5790,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -5774,7 +5799,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -5783,7 +5808,7 @@
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
@@ -5791,7 +5816,7 @@
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AD1" s="1"/>
       <c r="AE1" s="1"/>
@@ -5799,7 +5824,7 @@
       <c r="AG1" s="1"/>
       <c r="AH1" s="1"/>
       <c r="AI1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AJ1" s="1"/>
       <c r="AK1" s="1"/>
@@ -5819,16 +5844,16 @@
         <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>19</v>
@@ -5840,16 +5865,16 @@
         <v>21</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>19</v>
@@ -5861,16 +5886,16 @@
         <v>21</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>19</v>
@@ -5879,16 +5904,16 @@
         <v>20</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>19</v>
@@ -5897,16 +5922,16 @@
         <v>20</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AH2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AI2" s="1" t="s">
         <v>19</v>
@@ -5915,21 +5940,21 @@
         <v>20</v>
       </c>
       <c r="AK2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AL2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AM2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AN2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:40">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B3" s="1">
         <f>AVERAGE(Instances!B3:Instances!B12)</f>

</xml_diff>